<commit_message>
Informe dual  Ejercicio 2
</commit_message>
<xml_diff>
--- a/Taller_Dualidad_Solver_Completo.xlsx
+++ b/Taller_Dualidad_Solver_Completo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scavi\OneDrive\Documents\GitHub\ExcelSolverPL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leons\OneDrive\Desktop\Repos GIT\SolverExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6BC3613-EE52-4AE2-8A36-56EC50FB38EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC12218-38ED-4167-9650-A27ABBEE3F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E1 - Primal" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,11 @@
     <sheet name="E2 - Primal" sheetId="3" r:id="rId5"/>
     <sheet name="E2 - Informe Primal" sheetId="10" r:id="rId6"/>
     <sheet name="E2 - Dual" sheetId="4" r:id="rId7"/>
-    <sheet name="E3 - Primal" sheetId="5" r:id="rId8"/>
-    <sheet name="E3 - Dual" sheetId="6" r:id="rId9"/>
-    <sheet name="E4 - Primal" sheetId="7" r:id="rId10"/>
-    <sheet name="E4 - Dual" sheetId="8" r:id="rId11"/>
+    <sheet name="E2 - Informe Dual" sheetId="16" r:id="rId8"/>
+    <sheet name="E3 - Primal" sheetId="5" r:id="rId9"/>
+    <sheet name="E3 - Dual" sheetId="6" r:id="rId10"/>
+    <sheet name="E4 - Primal" sheetId="7" r:id="rId11"/>
+    <sheet name="E4 - Dual" sheetId="8" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="2" hidden="1">'E1 - Dual'!$B$2:$D$2</definedName>
@@ -181,7 +182,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="140">
   <si>
     <t>Variables</t>
   </si>
@@ -529,6 +530,78 @@
   </si>
   <si>
     <t>Iterations: 5 Subproblems: 0</t>
+  </si>
+  <si>
+    <t>Hoja de cálculo: [Taller_Dualidad_Solver_Completo.xlsx]E2 - Dual</t>
+  </si>
+  <si>
+    <t>Informe creado: 22/10/2026 11:35:28 a. m.</t>
+  </si>
+  <si>
+    <t>Iteraciones: 6 Subproblemas: 0</t>
+  </si>
+  <si>
+    <t>Celda objetivo (Mín)</t>
+  </si>
+  <si>
+    <t>$B$9</t>
+  </si>
+  <si>
+    <t>Z(min/max) Y1</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y1</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y2</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y3</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y4</t>
+  </si>
+  <si>
+    <t>$F$2</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y5</t>
+  </si>
+  <si>
+    <t>$G$2</t>
+  </si>
+  <si>
+    <t>Variables a encontrar Y6</t>
+  </si>
+  <si>
+    <t>$H$4</t>
+  </si>
+  <si>
+    <t>$H$4&gt;=$J$4</t>
+  </si>
+  <si>
+    <t>$H$5</t>
+  </si>
+  <si>
+    <t>$H$5&gt;=$J$5</t>
+  </si>
+  <si>
+    <t>$H$6</t>
+  </si>
+  <si>
+    <t>$H$6&gt;=$J$6</t>
+  </si>
+  <si>
+    <t>$H$7</t>
+  </si>
+  <si>
+    <t>R4 Recursos Utilizados</t>
+  </si>
+  <si>
+    <t>$H$7&gt;=$J$7</t>
+  </si>
+  <si>
+    <t>No vinculante</t>
   </si>
 </sst>
 </file>
@@ -672,7 +745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -687,21 +760,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1256,17 +1327,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
     <col min="2" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="9.21875" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1284,7 +1355,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1302,7 +1373,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1322,7 +1393,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1350,7 +1421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1378,7 +1449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1406,7 +1477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -1424,7 +1495,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1453,22 +1524,184 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="5" width="3" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
+        <f t="shared" ref="F4:F6" si="0">SUMPRODUCT($B$2:$E$2, B4:E4)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3">
+        <f t="shared" ref="I4:I6" si="1">H4-F4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2">
+        <f>SUMPRODUCT($B$2:$E$2, B7:E7)</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1486,7 +1719,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1498,7 +1731,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1518,7 +1751,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1536,7 +1769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1554,7 +1787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1572,7 +1805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -1584,7 +1817,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1604,23 +1837,23 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1638,7 +1871,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1650,7 +1883,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1670,7 +1903,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1688,7 +1921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1706,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1724,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -1736,7 +1969,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1759,280 +1992,274 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08FAB184-6C1B-49F8-B588-A22BFA1F04F8}">
   <dimension ref="A1:G32"/>
-  <sheetFormatPr defaultRowHeight="13.2" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.33203125" customWidth="1"/>
-    <col min="2" max="2" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="B6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
       <c r="B7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
       <c r="B8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:5" collapsed="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" collapsed="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="17" t="s">
+    <row r="15" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="9" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="14" t="s">
+    <row r="16" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="8">
         <v>18.658536585365855</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="8">
         <v>18.658536585365855</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="17" t="s">
+    <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="16" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-    </row>
-    <row r="22" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="13" t="s">
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="10">
         <v>2.1707317073170733</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="10">
         <v>2.1707317073170733</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="13" t="s">
+    <row r="23" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="10">
         <v>1.2195121951219514</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="10">
         <v>1.2195121951219514</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="13.8" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="14" t="s">
+    <row r="24" spans="1:7" ht="13.5" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="18">
+      <c r="D24" s="8">
         <v>1.5121951219512195</v>
       </c>
-      <c r="E24" s="18">
+      <c r="E24" s="8">
         <v>1.5121951219512195</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:7" collapsed="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="12"/>
-    </row>
-    <row r="28" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" collapsed="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="17" t="s">
+    <row r="29" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="10">
         <v>8</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G30" s="13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
+      <c r="G30" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="10">
         <v>10</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F31" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G31" s="13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="14" t="s">
+      <c r="G31" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="18">
+      <c r="D32" s="8">
         <v>15.000000000000002</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="F32" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="G32" s="14">
+      <c r="G32" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2047,17 +2274,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="25.33203125" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="26.6640625" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2075,7 +2302,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -2093,7 +2320,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -2113,7 +2340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -2139,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -2153,7 +2380,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="3">
-        <f t="shared" ref="E4:E6" si="1">SUMPRODUCT($B$2:$D$2, B5:D5)</f>
+        <f t="shared" ref="E5:E6" si="1">SUMPRODUCT($B$2:$D$2, B5:D5)</f>
         <v>5</v>
       </c>
       <c r="F5" s="3"/>
@@ -2165,7 +2392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -2191,7 +2418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -2209,7 +2436,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -2233,280 +2460,274 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6849234-CA33-4D5D-8C80-785D4BA712FD}">
   <dimension ref="A1:G32"/>
-  <sheetFormatPr defaultRowHeight="13.2" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.33203125" customWidth="1"/>
-    <col min="2" max="2" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="B6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
       <c r="B7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
       <c r="B8" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" collapsed="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:5" collapsed="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" collapsed="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="17" t="s">
+    <row r="15" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="9" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="14" t="s">
+    <row r="16" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D16" s="18">
-        <v>0</v>
-      </c>
-      <c r="E16" s="18">
+      <c r="D16" s="8">
+        <v>0</v>
+      </c>
+      <c r="E16" s="8">
         <v>18.658536585365855</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="17" t="s">
+    <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="16" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-    </row>
-    <row r="22" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="13" t="s">
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+    </row>
+    <row r="22" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D22" s="19">
-        <v>0</v>
-      </c>
-      <c r="E22" s="19">
+      <c r="D22" s="10">
+        <v>0</v>
+      </c>
+      <c r="E22" s="10">
         <v>1.0975609756097562</v>
       </c>
-      <c r="F22" s="13" t="s">
+      <c r="F22" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="13" t="s">
+    <row r="23" spans="1:7" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D23" s="19">
-        <v>0</v>
-      </c>
-      <c r="E23" s="19">
+      <c r="D23" s="10">
+        <v>0</v>
+      </c>
+      <c r="E23" s="10">
         <v>0.58536585365853666</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="F23" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="13.8" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="14" t="s">
+    <row r="24" spans="1:7" ht="13.5" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="18">
-        <v>0</v>
-      </c>
-      <c r="E24" s="18">
+      <c r="D24" s="8">
+        <v>0</v>
+      </c>
+      <c r="E24" s="8">
         <v>0.26829268292682917</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="8" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:7" collapsed="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="12"/>
-    </row>
-    <row r="28" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" collapsed="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="17" t="s">
+    <row r="29" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="17" t="s">
+      <c r="E29" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="17" t="s">
+      <c r="G29" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="10">
         <v>3</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="F30" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G30" s="19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
+      <c r="G30" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="10">
         <v>5</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F31" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="G31" s="19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="14" t="s">
+      <c r="G31" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D32" s="18">
+      <c r="D32" s="8">
         <v>4</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="F32" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="G32" s="18">
+      <c r="G32" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2521,19 +2742,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:K32"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="3" width="4.5546875" customWidth="1"/>
-    <col min="4" max="4" width="4.44140625" customWidth="1"/>
-    <col min="5" max="5" width="3.88671875" customWidth="1"/>
-    <col min="6" max="6" width="18.5546875" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="3" width="4.5703125" customWidth="1"/>
+    <col min="4" max="4" width="4.42578125" customWidth="1"/>
+    <col min="5" max="5" width="3.85546875" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2554,7 +2775,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -2575,7 +2796,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -2596,7 +2817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -2627,7 +2848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -2658,7 +2879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -2689,7 +2910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -2710,7 +2931,7 @@
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -2726,10 +2947,10 @@
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
     </row>
-    <row r="21" spans="8:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="8:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H21" s="4"/>
     </row>
-    <row r="32" spans="8:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="8:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K32" s="4"/>
     </row>
   </sheetData>
@@ -2741,81 +2962,81 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE75D373-4E18-420E-8661-9424F10D1AD8}">
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.33203125" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
       <c r="B6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
       <c r="B7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
       <c r="B8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
         <v>36</v>
       </c>
@@ -2829,7 +3050,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>46</v>
       </c>
@@ -2843,12 +3064,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B20" s="9" t="s">
         <v>36</v>
       </c>
@@ -2865,7 +3086,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B21" s="10" t="s">
         <v>48</v>
       </c>
@@ -2882,7 +3103,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B22" s="10" t="s">
         <v>51</v>
       </c>
@@ -2899,7 +3120,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B23" s="10" t="s">
         <v>53</v>
       </c>
@@ -2916,7 +3137,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>55</v>
       </c>
@@ -2933,12 +3154,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
         <v>36</v>
       </c>
@@ -2958,7 +3179,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B29" s="10" t="s">
         <v>57</v>
       </c>
@@ -2978,7 +3199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B30" s="10" t="s">
         <v>61</v>
       </c>
@@ -2998,7 +3219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
         <v>64</v>
       </c>
@@ -3029,22 +3250,22 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="2" width="4.140625" customWidth="1"/>
     <col min="3" max="3" width="3" customWidth="1"/>
     <col min="4" max="4" width="4" customWidth="1"/>
     <col min="5" max="5" width="3" customWidth="1"/>
     <col min="6" max="6" width="4" customWidth="1"/>
     <col min="7" max="7" width="3" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" customWidth="1"/>
-    <col min="10" max="10" width="17.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" customWidth="1"/>
     <col min="11" max="11" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3071,7 +3292,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3098,7 +3319,7 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -3121,7 +3342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -3156,7 +3377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -3191,7 +3412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -3226,7 +3447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -3261,7 +3482,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -3288,7 +3509,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -3313,22 +3534,364 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B477F4A1-9004-447D-A946-6977D22B5582}">
+  <dimension ref="A1:M35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="7"/>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="7"/>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="7"/>
+      <c r="B8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" s="17">
+        <v>15</v>
+      </c>
+      <c r="E16" s="17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="18">
+        <v>0</v>
+      </c>
+      <c r="E21" s="18">
+        <v>0</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D22" s="18">
+        <v>1</v>
+      </c>
+      <c r="E22" s="18">
+        <v>1</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B23" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="18">
+        <v>0</v>
+      </c>
+      <c r="E23" s="18">
+        <v>0</v>
+      </c>
+      <c r="F23" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="18">
+        <v>0</v>
+      </c>
+      <c r="E24" s="18">
+        <v>0</v>
+      </c>
+      <c r="F24" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B25" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="18">
+        <v>0</v>
+      </c>
+      <c r="E25" s="18">
+        <v>0</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="17">
+        <v>0</v>
+      </c>
+      <c r="E26" s="17">
+        <v>0</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="18">
+        <v>1</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G31" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B32" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="D32" s="18">
+        <v>2</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="F32" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G32" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B33" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="18">
+        <v>3</v>
+      </c>
+      <c r="E33" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G33" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="17">
+        <v>0</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="G34" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="M35" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
     <col min="2" max="4" width="3" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3346,7 +3909,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3358,7 +3921,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -3378,7 +3941,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -3396,7 +3959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -3414,7 +3977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -3432,7 +3995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -3450,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -3462,7 +4025,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -3480,166 +4043,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="5" width="3" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="10.44140625" customWidth="1"/>
-    <col min="8" max="8" width="17.44140625" customWidth="1"/>
-    <col min="9" max="9" width="7" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3">
-        <f t="shared" ref="F4:F6" si="0">SUMPRODUCT($B$2:$E$2, B4:E4)</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3">
-        <f t="shared" ref="I4:I6" si="1">H4-F4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2">
-        <f>SUMPRODUCT($B$2:$E$2, B7:E7)</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>